<commit_message>
aufgabe 1 am machen
</commit_message>
<xml_diff>
--- a/GP2/Versuch_O9/Mitschriften_O9.xlsx
+++ b/GP2/Versuch_O9/Mitschriften_O9.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fynnlucca/Documents/Grundpraktikum-1/GP2/Versuch_O9/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467708D9-EA7B-D944-8C62-221DEFC39F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785DE667-1F69-3D48-A9C6-6F04DCD88831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{5CCAB38F-6D57-5A42-BC81-AC9AC1713E20}"/>
+    <workbookView xWindow="11340" yWindow="1240" windowWidth="34560" windowHeight="20280" xr2:uid="{5CCAB38F-6D57-5A42-BC81-AC9AC1713E20}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>Versuch O9</t>
   </si>
@@ -96,6 +96,18 @@
   </si>
   <si>
     <t>Grün außen</t>
+  </si>
+  <si>
+    <t>durchschnitt</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>Abstand y</t>
+  </si>
+  <si>
+    <t>Abstand insgesamt</t>
   </si>
 </sst>
 </file>
@@ -467,15 +479,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A48620B9-AE64-8140-AFEB-AA4D4F9EA517}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -483,12 +495,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -513,8 +525,14 @@
       <c r="I7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
@@ -540,8 +558,16 @@
         <f>C8-F8</f>
         <v>767</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J8">
+        <f>D8-G8</f>
+        <v>3</v>
+      </c>
+      <c r="L8">
+        <f>SQRT(I8^2+J8^2)</f>
+        <v>767.00586699190251</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2</v>
       </c>
@@ -567,8 +593,16 @@
         <f t="shared" ref="I9:I11" si="0">C9-F9</f>
         <v>770</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J9">
+        <f t="shared" ref="J9:J11" si="1">D9-G9</f>
+        <v>6</v>
+      </c>
+      <c r="L9">
+        <f t="shared" ref="L9:L11" si="2">SQRT(I9^2+J9^2)</f>
+        <v>770.02337626853898</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>3</v>
       </c>
@@ -594,8 +628,16 @@
         <f t="shared" si="0"/>
         <v>763</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J10">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="2"/>
+        <v>763.02359072311776</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -621,18 +663,36 @@
         <f t="shared" si="0"/>
         <v>770</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J11">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="2"/>
+        <v>770.05259560630009</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G12">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14">
+        <f>AVERAGE(L8:L11)</f>
+        <v>767.52635739746484</v>
+      </c>
+      <c r="J14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -713,5 +773,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
aufgabe 1 fast feritg
</commit_message>
<xml_diff>
--- a/GP2/Versuch_O9/Mitschriften_O9.xlsx
+++ b/GP2/Versuch_O9/Mitschriften_O9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fynnlucca/Documents/Grundpraktikum-1/GP2/Versuch_O9/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785DE667-1F69-3D48-A9C6-6F04DCD88831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60952569-01C9-0849-BC36-07981A1CD59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11340" yWindow="1240" windowWidth="34560" windowHeight="20280" xr2:uid="{5CCAB38F-6D57-5A42-BC81-AC9AC1713E20}"/>
+    <workbookView xWindow="800" yWindow="2160" windowWidth="34560" windowHeight="20280" xr2:uid="{5CCAB38F-6D57-5A42-BC81-AC9AC1713E20}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>Versuch O9</t>
   </si>
@@ -108,6 +108,24 @@
   </si>
   <si>
     <t>Abstand insgesamt</t>
+  </si>
+  <si>
+    <t>Ring</t>
+  </si>
+  <si>
+    <t>Radius</t>
+  </si>
+  <si>
+    <t>Durchmesser</t>
+  </si>
+  <si>
+    <t>dunkle ringe</t>
+  </si>
+  <si>
+    <t>mm bis dreck</t>
+  </si>
+  <si>
+    <t>dreck bis ring</t>
   </si>
 </sst>
 </file>
@@ -479,15 +497,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A48620B9-AE64-8140-AFEB-AA4D4F9EA517}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -495,12 +518,54 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="Q4" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" t="s">
+        <v>25</v>
+      </c>
+      <c r="S4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P5" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>0.75</v>
+      </c>
+      <c r="S5">
+        <f>R5*2</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="O6">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="Q6">
+        <v>2</v>
+      </c>
+      <c r="R6">
+        <v>1.3169999999999999</v>
+      </c>
+      <c r="S6">
+        <f t="shared" ref="S6:S14" si="0">R6*2</f>
+        <v>2.6339999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -531,8 +596,21 @@
       <c r="L7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O7">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="Q7">
+        <v>3</v>
+      </c>
+      <c r="R7">
+        <v>1.6970000000000001</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="0"/>
+        <v>3.3940000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
@@ -566,8 +644,25 @@
         <f>SQRT(I8^2+J8^2)</f>
         <v>767.00586699190251</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O8">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P8">
+        <v>0.26300000000000001</v>
+      </c>
+      <c r="Q8">
+        <v>4</v>
+      </c>
+      <c r="R8">
+        <f>O6+P8</f>
+        <v>2.0379999999999998</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="0"/>
+        <v>4.0759999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2</v>
       </c>
@@ -590,19 +685,36 @@
         <v>965</v>
       </c>
       <c r="I9">
-        <f t="shared" ref="I9:I11" si="0">C9-F9</f>
+        <f t="shared" ref="I9:I11" si="1">C9-F9</f>
         <v>770</v>
       </c>
       <c r="J9">
-        <f t="shared" ref="J9:J11" si="1">D9-G9</f>
+        <f t="shared" ref="J9:J11" si="2">D9-G9</f>
         <v>6</v>
       </c>
       <c r="L9">
-        <f t="shared" ref="L9:L11" si="2">SQRT(I9^2+J9^2)</f>
+        <f t="shared" ref="L9:L11" si="3">SQRT(I9^2+J9^2)</f>
         <v>770.02337626853898</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O9">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P9">
+        <v>0.53400000000000003</v>
+      </c>
+      <c r="Q9">
+        <v>5</v>
+      </c>
+      <c r="R9">
+        <f>O6+P9</f>
+        <v>2.3090000000000002</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="0"/>
+        <v>4.6180000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>3</v>
       </c>
@@ -625,19 +737,36 @@
         <v>629</v>
       </c>
       <c r="I10">
+        <f t="shared" si="1"/>
+        <v>763</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="3"/>
+        <v>763.02359072311776</v>
+      </c>
+      <c r="O10">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P10">
+        <v>0.79500000000000004</v>
+      </c>
+      <c r="Q10">
+        <v>6</v>
+      </c>
+      <c r="R10">
+        <f t="shared" ref="R10" si="4">O8+P10</f>
+        <v>2.57</v>
+      </c>
+      <c r="S10">
         <f t="shared" si="0"/>
-        <v>763</v>
-      </c>
-      <c r="J10">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="L10">
-        <f t="shared" si="2"/>
-        <v>763.02359072311776</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -660,24 +789,77 @@
         <v>1704</v>
       </c>
       <c r="I11">
+        <f t="shared" si="1"/>
+        <v>770</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="3"/>
+        <v>770.05259560630009</v>
+      </c>
+      <c r="O11">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P11">
+        <v>1.0029999999999999</v>
+      </c>
+      <c r="Q11">
+        <v>7</v>
+      </c>
+      <c r="R11">
+        <f t="shared" ref="R11" si="5">O8+P11</f>
+        <v>2.7779999999999996</v>
+      </c>
+      <c r="S11">
         <f t="shared" si="0"/>
-        <v>770</v>
-      </c>
-      <c r="J11">
-        <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="L11">
-        <f t="shared" si="2"/>
-        <v>770.05259560630009</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+        <v>5.5559999999999992</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="G12">
         <v>78</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O12">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P12">
+        <v>1.214</v>
+      </c>
+      <c r="Q12">
+        <v>8</v>
+      </c>
+      <c r="R12">
+        <f t="shared" ref="R12" si="6">O10+P12</f>
+        <v>2.9889999999999999</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="0"/>
+        <v>5.9779999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="O13">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P13">
+        <v>1.407</v>
+      </c>
+      <c r="Q13">
+        <v>9</v>
+      </c>
+      <c r="R13">
+        <f t="shared" ref="R13" si="7">O10+P13</f>
+        <v>3.1819999999999999</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="0"/>
+        <v>6.3639999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -691,8 +873,44 @@
       <c r="J14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O14">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P14">
+        <v>1.5840000000000001</v>
+      </c>
+      <c r="Q14">
+        <v>10</v>
+      </c>
+      <c r="R14">
+        <f t="shared" ref="R14" si="8">O12+P14</f>
+        <v>3.359</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="0"/>
+        <v>6.718</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="O15">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="P15">
+        <v>1.764</v>
+      </c>
+      <c r="Q15">
+        <v>11</v>
+      </c>
+      <c r="R15">
+        <f t="shared" ref="R15" si="9">O12+P15</f>
+        <v>3.5389999999999997</v>
+      </c>
+      <c r="S15">
+        <f>R15*2</f>
+        <v>7.0779999999999994</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>9</v>
       </c>

</xml_diff>